<commit_message>
Atualiza planilha de implantação (sync automático)
</commit_message>
<xml_diff>
--- a/data/base/base implantação.xlsx
+++ b/data/base/base implantação.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mgcontecnica1-my.sharepoint.com/personal/warruda_mgcontecnica_com_br/Documents/Documentos/python/Portal-implantacao-tmp/data/base/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="582" documentId="11_4F56B3A8CB9C0E20059044E3BFE40D0DED129F61" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B302B61B-F6AF-4175-8BE1-1778158AB9FF}"/>
+  <xr:revisionPtr revIDLastSave="607" documentId="11_4F56B3A8CB9C0E20059044E3BFE40D0DED129F61" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{73EC1ED9-1A89-48FE-8703-CD14F37C8ACE}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="544" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="534" uniqueCount="234">
   <si>
     <t>ID</t>
   </si>
@@ -564,9 +564,6 @@
   </si>
   <si>
     <t>AA&amp;amp;MARTINS PARTICIPACOES LTDA ;ADRIANO AUGUSTO MARTINS ;E&amp;amp;G MARTINS PARTICIPACOES LTDA ;EDUARDO DE JESUS MARTINS  ; B&amp;amp;SOLAR PARTICIPACOES LTDA ;MARCOS MARQUES MARTINS ;</t>
-  </si>
-  <si>
-    <t>Karina Santos</t>
   </si>
   <si>
     <t>COMERCIO VAREJISTA DE MERCADORIAS 3M LTDA (FILIAL 1)</t>
@@ -1890,7 +1887,7 @@
         <v>54</v>
       </c>
       <c r="N4" s="9">
-        <v>46232</v>
+        <v>46290</v>
       </c>
       <c r="O4" s="5" t="s">
         <v>39</v>
@@ -1951,8 +1948,8 @@
       <c r="M5" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="N5" s="8">
-        <v>46232</v>
+      <c r="N5" s="9">
+        <v>46290</v>
       </c>
       <c r="O5" s="7" t="s">
         <v>39</v>
@@ -3145,9 +3142,7 @@
       <c r="O23" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="P23" s="7" t="s">
-        <v>176</v>
-      </c>
+      <c r="P23" s="7"/>
       <c r="Q23" s="7"/>
       <c r="R23" s="7"/>
       <c r="S23" s="7"/>
@@ -3170,7 +3165,7 @@
         <v>7012</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C24" s="5">
         <v>46235</v>
@@ -3191,7 +3186,7 @@
         <v>102</v>
       </c>
       <c r="I24" s="5" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="J24" s="5" t="s">
         <v>173</v>
@@ -3203,7 +3198,7 @@
         <v>64</v>
       </c>
       <c r="M24" s="5" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="N24" s="20">
         <v>46255</v>
@@ -3211,9 +3206,7 @@
       <c r="O24" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="P24" s="7" t="s">
-        <v>176</v>
-      </c>
+      <c r="P24" s="5"/>
       <c r="Q24" s="5"/>
       <c r="R24" s="5"/>
       <c r="S24" s="5"/>
@@ -3236,7 +3229,7 @@
         <v>7014</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C25" s="7">
         <v>46235</v>
@@ -3257,19 +3250,19 @@
         <v>93</v>
       </c>
       <c r="I25" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="J25" s="7" t="s">
         <v>181</v>
       </c>
-      <c r="J25" s="7" t="s">
+      <c r="K25" s="7" t="s">
         <v>182</v>
       </c>
-      <c r="K25" s="7" t="s">
+      <c r="L25" s="7" t="s">
         <v>183</v>
       </c>
-      <c r="L25" s="7" t="s">
+      <c r="M25" s="7" t="s">
         <v>184</v>
-      </c>
-      <c r="M25" s="7" t="s">
-        <v>185</v>
       </c>
       <c r="N25" s="20">
         <v>46255</v>
@@ -3277,9 +3270,7 @@
       <c r="O25" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="P25" s="7" t="s">
-        <v>176</v>
-      </c>
+      <c r="P25" s="7"/>
       <c r="Q25" s="7"/>
       <c r="R25" s="7"/>
       <c r="S25" s="7"/>
@@ -3302,7 +3293,7 @@
         <v>7015</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C26" s="5">
         <v>46235</v>
@@ -3323,10 +3314,10 @@
         <v>93</v>
       </c>
       <c r="I26" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="J26" s="5" t="s">
         <v>187</v>
-      </c>
-      <c r="J26" s="5" t="s">
-        <v>188</v>
       </c>
       <c r="K26" s="5" t="s">
         <v>174</v>
@@ -3335,7 +3326,7 @@
         <v>64</v>
       </c>
       <c r="M26" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="N26" s="20">
         <v>46255</v>
@@ -3343,9 +3334,7 @@
       <c r="O26" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="P26" s="7" t="s">
-        <v>176</v>
-      </c>
+      <c r="P26" s="5"/>
       <c r="Q26" s="5"/>
       <c r="R26" s="5"/>
       <c r="S26" s="5"/>
@@ -3368,7 +3357,7 @@
         <v>7016</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C27" s="7">
         <v>46235</v>
@@ -3377,10 +3366,10 @@
         <v>169</v>
       </c>
       <c r="E27" s="7" t="s">
+        <v>190</v>
+      </c>
+      <c r="F27" s="7" t="s">
         <v>191</v>
-      </c>
-      <c r="F27" s="7" t="s">
-        <v>192</v>
       </c>
       <c r="G27" s="7" t="s">
         <v>150</v>
@@ -3389,19 +3378,19 @@
         <v>93</v>
       </c>
       <c r="I27" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="J27" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="K27" s="7" t="s">
         <v>193</v>
       </c>
-      <c r="J27" s="7" t="s">
-        <v>182</v>
-      </c>
-      <c r="K27" s="7" t="s">
+      <c r="L27" s="7" t="s">
+        <v>183</v>
+      </c>
+      <c r="M27" s="7" t="s">
         <v>194</v>
-      </c>
-      <c r="L27" s="7" t="s">
-        <v>184</v>
-      </c>
-      <c r="M27" s="7" t="s">
-        <v>195</v>
       </c>
       <c r="N27" s="20">
         <v>46255</v>
@@ -3409,9 +3398,7 @@
       <c r="O27" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="P27" s="7" t="s">
-        <v>176</v>
-      </c>
+      <c r="P27" s="7"/>
       <c r="Q27" s="7"/>
       <c r="R27" s="7"/>
       <c r="S27" s="7"/>
@@ -3434,7 +3421,7 @@
         <v>7017</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C28" s="5">
         <v>46235</v>
@@ -3455,7 +3442,7 @@
         <v>93</v>
       </c>
       <c r="I28" s="5" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="J28" s="5" t="s">
         <v>173</v>
@@ -3467,7 +3454,7 @@
         <v>64</v>
       </c>
       <c r="M28" s="5" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="N28" s="20">
         <v>46255</v>
@@ -3475,9 +3462,7 @@
       <c r="O28" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="P28" s="7" t="s">
-        <v>176</v>
-      </c>
+      <c r="P28" s="5"/>
       <c r="Q28" s="5"/>
       <c r="R28" s="5"/>
       <c r="S28" s="5"/>
@@ -3500,7 +3485,7 @@
         <v>7018</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C29" s="7">
         <v>46235</v>
@@ -3509,10 +3494,10 @@
         <v>169</v>
       </c>
       <c r="E29" s="7" t="s">
+        <v>190</v>
+      </c>
+      <c r="F29" s="7" t="s">
         <v>191</v>
-      </c>
-      <c r="F29" s="7" t="s">
-        <v>192</v>
       </c>
       <c r="G29" s="7" t="s">
         <v>150</v>
@@ -3521,7 +3506,7 @@
         <v>93</v>
       </c>
       <c r="I29" s="7" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="J29" s="7" t="s">
         <v>173</v>
@@ -3533,7 +3518,7 @@
         <v>64</v>
       </c>
       <c r="M29" s="7" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="N29" s="20">
         <v>46255</v>
@@ -3541,9 +3526,7 @@
       <c r="O29" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="P29" s="7" t="s">
-        <v>176</v>
-      </c>
+      <c r="P29" s="7"/>
       <c r="Q29" s="7"/>
       <c r="R29" s="7"/>
       <c r="S29" s="7"/>
@@ -3566,7 +3549,7 @@
         <v>7019</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C30" s="5">
         <v>46235</v>
@@ -3587,10 +3570,10 @@
         <v>93</v>
       </c>
       <c r="I30" s="5" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="J30" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="K30" s="5" t="s">
         <v>174</v>
@@ -3599,7 +3582,7 @@
         <v>64</v>
       </c>
       <c r="M30" s="5" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="N30" s="20">
         <v>46255</v>
@@ -3607,9 +3590,7 @@
       <c r="O30" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="P30" s="7" t="s">
-        <v>176</v>
-      </c>
+      <c r="P30" s="5"/>
       <c r="Q30" s="5"/>
       <c r="R30" s="5"/>
       <c r="S30" s="5"/>
@@ -3632,7 +3613,7 @@
         <v>7020</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C31" s="7">
         <v>46235</v>
@@ -3653,19 +3634,19 @@
         <v>93</v>
       </c>
       <c r="I31" s="7" t="s">
+        <v>199</v>
+      </c>
+      <c r="J31" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="K31" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="L31" s="7" t="s">
+        <v>183</v>
+      </c>
+      <c r="M31" s="7" t="s">
         <v>200</v>
-      </c>
-      <c r="J31" s="7" t="s">
-        <v>182</v>
-      </c>
-      <c r="K31" s="7" t="s">
-        <v>194</v>
-      </c>
-      <c r="L31" s="7" t="s">
-        <v>184</v>
-      </c>
-      <c r="M31" s="7" t="s">
-        <v>201</v>
       </c>
       <c r="N31" s="20">
         <v>46255</v>
@@ -3673,9 +3654,7 @@
       <c r="O31" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="P31" s="7" t="s">
-        <v>176</v>
-      </c>
+      <c r="P31" s="7"/>
       <c r="Q31" s="7"/>
       <c r="R31" s="7"/>
       <c r="S31" s="7"/>
@@ -3698,7 +3677,7 @@
         <v>7021</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C32" s="5">
         <v>46235</v>
@@ -3707,10 +3686,10 @@
         <v>169</v>
       </c>
       <c r="E32" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="F32" s="5" t="s">
         <v>191</v>
-      </c>
-      <c r="F32" s="5" t="s">
-        <v>192</v>
       </c>
       <c r="G32" s="5" t="s">
         <v>150</v>
@@ -3719,19 +3698,19 @@
         <v>93</v>
       </c>
       <c r="I32" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="J32" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="K32" s="5" t="s">
         <v>193</v>
       </c>
-      <c r="J32" s="5" t="s">
-        <v>182</v>
-      </c>
-      <c r="K32" s="5" t="s">
-        <v>194</v>
-      </c>
       <c r="L32" s="5" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="M32" s="5" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="N32" s="20">
         <v>46255</v>
@@ -3739,9 +3718,7 @@
       <c r="O32" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="P32" s="7" t="s">
-        <v>176</v>
-      </c>
+      <c r="P32" s="5"/>
       <c r="Q32" s="5"/>
       <c r="R32" s="5"/>
       <c r="S32" s="5"/>
@@ -3764,16 +3741,16 @@
         <v>6992</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C33" s="7">
         <v>46266</v>
       </c>
       <c r="D33" s="7" t="s">
+        <v>203</v>
+      </c>
+      <c r="E33" s="7" t="s">
         <v>204</v>
-      </c>
-      <c r="E33" s="7" t="s">
-        <v>205</v>
       </c>
       <c r="F33" s="7" t="s">
         <v>149</v>
@@ -3785,19 +3762,19 @@
         <v>102</v>
       </c>
       <c r="I33" s="7" t="s">
+        <v>205</v>
+      </c>
+      <c r="J33" s="7" t="s">
         <v>206</v>
       </c>
-      <c r="J33" s="7" t="s">
+      <c r="K33" s="7" t="s">
         <v>207</v>
-      </c>
-      <c r="K33" s="7" t="s">
-        <v>208</v>
       </c>
       <c r="L33" s="7" t="s">
         <v>64</v>
       </c>
       <c r="M33" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="N33" s="7"/>
       <c r="O33" s="7" t="s">
@@ -3828,16 +3805,16 @@
         <v>6993</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C34" s="5">
         <v>46266</v>
       </c>
       <c r="D34" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="E34" s="5" t="s">
         <v>204</v>
-      </c>
-      <c r="E34" s="5" t="s">
-        <v>205</v>
       </c>
       <c r="F34" s="5" t="s">
         <v>149</v>
@@ -3849,19 +3826,19 @@
         <v>33</v>
       </c>
       <c r="I34" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="J34" s="5" t="s">
         <v>211</v>
       </c>
-      <c r="J34" s="5" t="s">
+      <c r="K34" s="5" t="s">
         <v>212</v>
-      </c>
-      <c r="K34" s="5" t="s">
-        <v>213</v>
       </c>
       <c r="L34" s="5" t="s">
         <v>64</v>
       </c>
       <c r="M34" s="5" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="N34" s="5"/>
       <c r="O34" s="5" t="s">
@@ -3892,13 +3869,13 @@
         <v>6945</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C35" s="7">
         <v>46174</v>
       </c>
       <c r="D35" s="7" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="E35" s="7" t="s">
         <v>148</v>
@@ -3913,19 +3890,19 @@
         <v>33</v>
       </c>
       <c r="I35" s="13" t="s">
+        <v>216</v>
+      </c>
+      <c r="J35" s="7" t="s">
         <v>217</v>
       </c>
-      <c r="J35" s="7" t="s">
+      <c r="K35" s="7" t="s">
         <v>218</v>
-      </c>
-      <c r="K35" s="7" t="s">
-        <v>219</v>
       </c>
       <c r="L35" s="7" t="s">
         <v>37</v>
       </c>
       <c r="M35" s="7" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="N35" s="8">
         <v>46219</v>
@@ -3960,19 +3937,19 @@
         <v>7036</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C36" s="5">
         <v>46266</v>
       </c>
       <c r="D36" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="E36" s="5" t="s">
         <v>222</v>
       </c>
-      <c r="E36" s="5" t="s">
+      <c r="F36" s="5" t="s">
         <v>223</v>
-      </c>
-      <c r="F36" s="5" t="s">
-        <v>224</v>
       </c>
       <c r="G36" s="5" t="s">
         <v>150</v>
@@ -3981,32 +3958,32 @@
         <v>102</v>
       </c>
       <c r="I36" s="5" t="s">
+        <v>224</v>
+      </c>
+      <c r="J36" s="5" t="s">
         <v>225</v>
       </c>
-      <c r="J36" s="5" t="s">
+      <c r="K36" s="5" t="s">
         <v>226</v>
-      </c>
-      <c r="K36" s="5" t="s">
-        <v>227</v>
       </c>
       <c r="L36" s="5" t="s">
         <v>64</v>
       </c>
       <c r="M36" s="5" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="N36" s="5"/>
       <c r="O36" s="5" t="s">
         <v>39</v>
       </c>
       <c r="P36" s="5" t="s">
+        <v>228</v>
+      </c>
+      <c r="Q36" s="5" t="s">
         <v>229</v>
       </c>
-      <c r="Q36" s="5" t="s">
+      <c r="R36" s="5" t="s">
         <v>230</v>
-      </c>
-      <c r="R36" s="5" t="s">
-        <v>231</v>
       </c>
       <c r="S36" s="5"/>
       <c r="T36" s="5" t="s">
@@ -4028,19 +4005,19 @@
         <v>7037</v>
       </c>
       <c r="B37" s="15" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C37" s="15">
         <v>46266</v>
       </c>
       <c r="D37" s="15" t="s">
+        <v>221</v>
+      </c>
+      <c r="E37" s="15" t="s">
         <v>222</v>
       </c>
-      <c r="E37" s="15" t="s">
+      <c r="F37" s="15" t="s">
         <v>223</v>
-      </c>
-      <c r="F37" s="15" t="s">
-        <v>224</v>
       </c>
       <c r="G37" s="15" t="s">
         <v>150</v>
@@ -4049,32 +4026,32 @@
         <v>33</v>
       </c>
       <c r="I37" s="15" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="J37" s="15" t="s">
+        <v>225</v>
+      </c>
+      <c r="K37" s="15" t="s">
         <v>226</v>
-      </c>
-      <c r="K37" s="15" t="s">
-        <v>227</v>
       </c>
       <c r="L37" s="15" t="s">
         <v>64</v>
       </c>
       <c r="M37" s="15" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="N37" s="15"/>
       <c r="O37" s="15" t="s">
         <v>39</v>
       </c>
       <c r="P37" s="7" t="s">
+        <v>228</v>
+      </c>
+      <c r="Q37" s="7" t="s">
         <v>229</v>
       </c>
-      <c r="Q37" s="7" t="s">
+      <c r="R37" s="19" t="s">
         <v>230</v>
-      </c>
-      <c r="R37" s="19" t="s">
-        <v>231</v>
       </c>
       <c r="S37" s="15"/>
       <c r="T37" s="15" t="s">

</xml_diff>